<commit_message>
Added in a new batch crafting automation. Added in new logging and location templates
</commit_message>
<xml_diff>
--- a/resources/data-imports/World Gems/map-gems.xlsx
+++ b/resources/data-imports/World Gems/map-gems.xlsx
@@ -7,15 +7,15 @@
     <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Map Gems" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="67">
   <si>
     <t>id</t>
   </si>
@@ -128,61 +128,94 @@
     <t>monster_atonement_range</t>
   </si>
   <si>
-    <t>Shadow Of Illusion</t>
-  </si>
-  <si>
-    <t>The shadows of the past, the present and the future - a yet untold tale - all intertwind and make an illusion of what never was.</t>
+    <t>Shadow Plane Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for Shadow Plane after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
   </si>
   <si>
     <t>Shadow Plane</t>
   </si>
   <si>
-    <t>Alchemy</t>
-  </si>
-  <si>
-    <t>0.05-0.012</t>
-  </si>
-  <si>
-    <t>0.02-0.08</t>
-  </si>
-  <si>
-    <t>0.08-0.12</t>
-  </si>
-  <si>
-    <t>0.08-0.16</t>
-  </si>
-  <si>
-    <t>0.03-0.11</t>
-  </si>
-  <si>
-    <t>0.05-0.16</t>
-  </si>
-  <si>
-    <t>0.05-0.10</t>
-  </si>
-  <si>
-    <t>0.08-0.13</t>
-  </si>
-  <si>
-    <t>0.08-0.10</t>
-  </si>
-  <si>
-    <t>0.08-0.20</t>
-  </si>
-  <si>
     <t>0.08-0.15</t>
   </si>
   <si>
-    <t>0.03-0.10</t>
-  </si>
-  <si>
-    <t>0.03-0.15</t>
-  </si>
-  <si>
-    <t>0.03-0.18</t>
-  </si>
-  <si>
-    <t>1.00-3.00</t>
+    <t>0.04-0.12</t>
+  </si>
+  <si>
+    <t>0.06-0.12</t>
+  </si>
+  <si>
+    <t>Hell Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for Hell after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
+  </si>
+  <si>
+    <t>Hell</t>
+  </si>
+  <si>
+    <t>0.12-0.2</t>
+  </si>
+  <si>
+    <t>0.2-0.3</t>
+  </si>
+  <si>
+    <t>0.18-0.25</t>
+  </si>
+  <si>
+    <t>Purgatory Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for Purgatory after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
+  </si>
+  <si>
+    <t>Purgatory</t>
+  </si>
+  <si>
+    <t>0.25-0.38</t>
+  </si>
+  <si>
+    <t>0.28-0.39</t>
+  </si>
+  <si>
+    <t>0.3-0.55</t>
+  </si>
+  <si>
+    <t>Twisted Memories Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for Twisted Memories after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
+  </si>
+  <si>
+    <t>Twisted Memories</t>
+  </si>
+  <si>
+    <t>0.35-0.43</t>
+  </si>
+  <si>
+    <t>0.42-0.48</t>
+  </si>
+  <si>
+    <t>0.48-0.65</t>
+  </si>
+  <si>
+    <t>Delusional Memories Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for Delusional Memories after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
+  </si>
+  <si>
+    <t>Delusional Memories</t>
+  </si>
+  <si>
+    <t>The Ice Plane Gem Profile</t>
+  </si>
+  <si>
+    <t>Gem profile for The Ice Plane after the Federation devastation and the Childs unstable memory reshaped its rewards.</t>
+  </si>
+  <si>
+    <t>The Ice Plane</t>
   </si>
 </sst>
 </file>
@@ -522,47 +555,8 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AK7"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="3.428" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="152.106" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="42.418" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="48.274" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="47.131" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="37.705" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="45.846" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="45.846" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="45.846" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="48.274" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="37.705" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="26" max="26" width="41.133" bestFit="true" customWidth="true" style="0"/>
-    <col min="27" max="27" width="44.703" bestFit="true" customWidth="true" style="0"/>
-    <col min="28" max="28" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="29" max="29" width="35.277" bestFit="true" customWidth="true" style="0"/>
-    <col min="30" max="30" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="31" max="31" width="36.42" bestFit="true" customWidth="true" style="0"/>
-    <col min="32" max="32" width="51.845" bestFit="true" customWidth="true" style="0"/>
-    <col min="33" max="33" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="34" max="34" width="38.848" bestFit="true" customWidth="true" style="0"/>
-    <col min="35" max="35" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="36" max="36" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="37" max="37" width="28.136" bestFit="true" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:37">
       <c r="A1" t="s">
@@ -678,9 +672,6 @@
       </c>
     </row>
     <row r="2" spans="1:37">
-      <c r="A2">
-        <v>1</v>
-      </c>
       <c r="B2" t="s">
         <v>37</v>
       </c>
@@ -690,68 +681,618 @@
       <c r="D2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N2" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
         <v>41</v>
       </c>
-      <c r="G2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="U2" t="s">
+        <v>42</v>
+      </c>
+      <c r="V2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37">
+      <c r="B3" t="s">
         <v>43</v>
       </c>
-      <c r="J2" t="s">
+      <c r="C3" t="s">
         <v>44</v>
       </c>
-      <c r="K2" t="s">
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="M2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="F3" t="s">
         <v>46</v>
       </c>
-      <c r="O2" t="s">
+      <c r="G3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" t="s">
+        <v>46</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" t="s">
+        <v>46</v>
+      </c>
+      <c r="O3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
         <v>47</v>
       </c>
-      <c r="T2" t="s">
-        <v>48</v>
-      </c>
-      <c r="U2" t="s">
+      <c r="U3" t="s">
+        <v>48</v>
+      </c>
+      <c r="V3" t="s">
+        <v>48</v>
+      </c>
+      <c r="W3" t="s">
+        <v>48</v>
+      </c>
+      <c r="X3" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:37">
+      <c r="B4" t="s">
         <v>49</v>
       </c>
-      <c r="V2" t="s">
-        <v>44</v>
-      </c>
-      <c r="W2" t="s">
-        <v>44</v>
-      </c>
-      <c r="X2" t="s">
+      <c r="C4" t="s">
         <v>50</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="D4" t="s">
         <v>51</v>
       </c>
-      <c r="Z2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>52</v>
-      </c>
-      <c r="AG2" t="s">
+      <c r="F4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" t="s">
+        <v>52</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4" t="s">
         <v>53</v>
       </c>
-      <c r="AH2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AI2" t="s">
+      <c r="U4" t="s">
+        <v>54</v>
+      </c>
+      <c r="V4" t="s">
+        <v>54</v>
+      </c>
+      <c r="W4" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:37">
+      <c r="B5" t="s">
         <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" t="s">
+        <v>58</v>
+      </c>
+      <c r="M5" t="s">
+        <v>58</v>
+      </c>
+      <c r="N5" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" t="s">
+        <v>58</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5" t="s">
+        <v>59</v>
+      </c>
+      <c r="U5" t="s">
+        <v>60</v>
+      </c>
+      <c r="V5" t="s">
+        <v>60</v>
+      </c>
+      <c r="W5" t="s">
+        <v>60</v>
+      </c>
+      <c r="X5" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37">
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M6" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" t="s">
+        <v>58</v>
+      </c>
+      <c r="O6" t="s">
+        <v>58</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6" t="s">
+        <v>59</v>
+      </c>
+      <c r="U6" t="s">
+        <v>60</v>
+      </c>
+      <c r="V6" t="s">
+        <v>60</v>
+      </c>
+      <c r="W6" t="s">
+        <v>60</v>
+      </c>
+      <c r="X6" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37">
+      <c r="B7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" t="s">
+        <v>52</v>
+      </c>
+      <c r="M7" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7" t="s">
+        <v>52</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7" t="s">
+        <v>53</v>
+      </c>
+      <c r="U7" t="s">
+        <v>54</v>
+      </c>
+      <c r="V7" t="s">
+        <v>54</v>
+      </c>
+      <c r="W7" t="s">
+        <v>54</v>
+      </c>
+      <c r="X7" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>